<commit_message>
last last last fix
</commit_message>
<xml_diff>
--- a/dados-tratados.xlsx
+++ b/dados-tratados.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Desktop\TESTE-ANALISTA-SBF\excel_pandas\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Desktop\TESTE-ANALISTA-SBF\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4CF11358-1689-4BA1-B14A-E7B8D298E3F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59D5D9A6-E80C-4F0C-A52A-0DC72751A7A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="2" r:id="rId1"/>

</xml_diff>